<commit_message>
Split two Faro scene headers out of dialogue lines; refresh workbook positions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7XwMhLTxaQujwLWpYAxgB
</commit_message>
<xml_diff>
--- a/알바로_부작_화_목록.xlsx
+++ b/알바로_부작_화_목록.xlsx
@@ -21279,7 +21279,7 @@
         <v>11941</v>
       </c>
       <c r="F657" s="13" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G657" s="15" t="inlineStr">
         <is>
@@ -21304,10 +21304,10 @@
         </is>
       </c>
       <c r="E658" s="13" t="n">
-        <v>12008</v>
+        <v>12005</v>
       </c>
       <c r="F658" s="13" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G658" s="15" t="inlineStr">
         <is>
@@ -21332,10 +21332,10 @@
         </is>
       </c>
       <c r="E659" s="13" t="n">
-        <v>12029</v>
+        <v>12032</v>
       </c>
       <c r="F659" s="13" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G659" s="15" t="inlineStr">
         <is>
@@ -21360,7 +21360,7 @@
         </is>
       </c>
       <c r="E660" s="13" t="n">
-        <v>12073</v>
+        <v>12075</v>
       </c>
       <c r="F660" s="13" t="n">
         <v>47</v>
@@ -21388,7 +21388,7 @@
         </is>
       </c>
       <c r="E661" s="13" t="n">
-        <v>12125</v>
+        <v>12127</v>
       </c>
       <c r="F661" s="13" t="n">
         <v>40</v>
@@ -21416,7 +21416,7 @@
         </is>
       </c>
       <c r="E662" s="13" t="n">
-        <v>12169</v>
+        <v>12171</v>
       </c>
       <c r="F662" s="13" t="n">
         <v>14</v>
@@ -21444,7 +21444,7 @@
         </is>
       </c>
       <c r="E663" s="13" t="n">
-        <v>12185</v>
+        <v>12187</v>
       </c>
       <c r="F663" s="13" t="n">
         <v>12</v>
@@ -21472,7 +21472,7 @@
         </is>
       </c>
       <c r="E664" s="13" t="n">
-        <v>12200</v>
+        <v>12202</v>
       </c>
       <c r="F664" s="13" t="n">
         <v>12</v>
@@ -21500,7 +21500,7 @@
         </is>
       </c>
       <c r="E665" s="13" t="n">
-        <v>12215</v>
+        <v>12217</v>
       </c>
       <c r="F665" s="13" t="n">
         <v>12</v>
@@ -21528,7 +21528,7 @@
         </is>
       </c>
       <c r="E666" s="13" t="n">
-        <v>12230</v>
+        <v>12232</v>
       </c>
       <c r="F666" s="13" t="n">
         <v>12</v>
@@ -21556,7 +21556,7 @@
         </is>
       </c>
       <c r="E667" s="13" t="n">
-        <v>12244</v>
+        <v>12246</v>
       </c>
       <c r="F667" s="13" t="n">
         <v>12</v>
@@ -21584,7 +21584,7 @@
         </is>
       </c>
       <c r="E668" s="13" t="n">
-        <v>12258</v>
+        <v>12260</v>
       </c>
       <c r="F668" s="13" t="n">
         <v>10</v>
@@ -21612,10 +21612,10 @@
         </is>
       </c>
       <c r="E669" s="13" t="n">
-        <v>12271</v>
+        <v>12273</v>
       </c>
       <c r="F669" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G669" s="15" t="inlineStr">
         <is>
@@ -21640,7 +21640,7 @@
         </is>
       </c>
       <c r="E670" s="13" t="n">
-        <v>12287</v>
+        <v>12288</v>
       </c>
       <c r="F670" s="13" t="n">
         <v>12</v>
@@ -21668,7 +21668,7 @@
         </is>
       </c>
       <c r="E671" s="13" t="n">
-        <v>12301</v>
+        <v>12302</v>
       </c>
       <c r="F671" s="13" t="n">
         <v>13</v>
@@ -21696,10 +21696,10 @@
         </is>
       </c>
       <c r="E672" s="13" t="n">
-        <v>12316</v>
+        <v>12317</v>
       </c>
       <c r="F672" s="13" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G672" s="15" t="inlineStr">
         <is>
@@ -21727,7 +21727,7 @@
         <v>12398</v>
       </c>
       <c r="F673" s="13" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G673" s="15" t="inlineStr">
         <is>
@@ -21752,10 +21752,10 @@
         </is>
       </c>
       <c r="E674" s="13" t="n">
-        <v>12528</v>
+        <v>12527</v>
       </c>
       <c r="F674" s="13" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G674" s="15" t="inlineStr">
         <is>
@@ -21780,10 +21780,10 @@
         </is>
       </c>
       <c r="E675" s="13" t="n">
-        <v>12578</v>
+        <v>12576</v>
       </c>
       <c r="F675" s="13" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G675" s="15" t="inlineStr">
         <is>
@@ -21808,10 +21808,10 @@
         </is>
       </c>
       <c r="E676" s="13" t="n">
-        <v>12648</v>
+        <v>12643</v>
       </c>
       <c r="F676" s="13" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G676" s="15" t="inlineStr">
         <is>
@@ -21836,10 +21836,10 @@
         </is>
       </c>
       <c r="E677" s="13" t="n">
-        <v>12707</v>
+        <v>12700</v>
       </c>
       <c r="F677" s="13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G677" s="15" t="inlineStr">
         <is>
@@ -21864,10 +21864,10 @@
         </is>
       </c>
       <c r="E678" s="13" t="n">
-        <v>12718</v>
+        <v>12713</v>
       </c>
       <c r="F678" s="13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G678" s="15" t="inlineStr">
         <is>
@@ -21892,7 +21892,7 @@
         </is>
       </c>
       <c r="E679" s="13" t="n">
-        <v>12732</v>
+        <v>12726</v>
       </c>
       <c r="F679" s="13" t="n">
         <v>9</v>
@@ -21920,7 +21920,7 @@
         </is>
       </c>
       <c r="E680" s="13" t="n">
-        <v>12743</v>
+        <v>12737</v>
       </c>
       <c r="F680" s="13" t="n">
         <v>26</v>
@@ -21948,10 +21948,10 @@
         </is>
       </c>
       <c r="E681" s="13" t="n">
-        <v>12773</v>
+        <v>12767</v>
       </c>
       <c r="F681" s="13" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G681" s="15" t="inlineStr">
         <is>
@@ -21976,7 +21976,7 @@
         </is>
       </c>
       <c r="E682" s="13" t="n">
-        <v>12804</v>
+        <v>12796</v>
       </c>
       <c r="F682" s="13" t="n">
         <v>18</v>
@@ -22004,10 +22004,10 @@
         </is>
       </c>
       <c r="E683" s="13" t="n">
-        <v>12825</v>
+        <v>12817</v>
       </c>
       <c r="F683" s="13" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G683" s="15" t="inlineStr">
         <is>
@@ -22032,7 +22032,7 @@
         </is>
       </c>
       <c r="E684" s="13" t="n">
-        <v>12851</v>
+        <v>12842</v>
       </c>
       <c r="F684" s="13" t="n">
         <v>19</v>
@@ -22060,10 +22060,10 @@
         </is>
       </c>
       <c r="E685" s="13" t="n">
-        <v>12873</v>
+        <v>12864</v>
       </c>
       <c r="F685" s="13" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G685" s="15" t="inlineStr">
         <is>
@@ -22088,7 +22088,7 @@
         </is>
       </c>
       <c r="E686" s="13" t="n">
-        <v>12898</v>
+        <v>12888</v>
       </c>
       <c r="F686" s="13" t="n">
         <v>18</v>
@@ -22116,7 +22116,7 @@
         </is>
       </c>
       <c r="E687" s="13" t="n">
-        <v>12919</v>
+        <v>12909</v>
       </c>
       <c r="F687" s="13" t="n">
         <v>18</v>
@@ -22144,7 +22144,7 @@
         </is>
       </c>
       <c r="E688" s="13" t="n">
-        <v>12940</v>
+        <v>12930</v>
       </c>
       <c r="F688" s="13" t="n">
         <v>17</v>
@@ -22172,7 +22172,7 @@
         </is>
       </c>
       <c r="E689" s="13" t="n">
-        <v>12960</v>
+        <v>12950</v>
       </c>
       <c r="F689" s="13" t="n">
         <v>11</v>
@@ -22200,14 +22200,14 @@
         </is>
       </c>
       <c r="E690" s="13" t="n">
-        <v>12973</v>
+        <v>12963</v>
       </c>
       <c r="F690" s="13" t="n">
         <v>18</v>
       </c>
       <c r="G690" s="15" t="inlineStr">
         <is>
-          <t>새로운 세션. 빅토르가 '마레아 작전'을 설명합니다 — 북방의 교향곡과 바벨탑이 인프라라면, 마레아는 특정 선거를 겨냥해 그 인프라 전체를 가동시키는 실행 단계입니다. 특정 정당이나 후 보는 언급하지 않고, 기법 자체에 초점을 맞춥니다.</t>
+          <t>새로운 세션. 빅토르가 '마레아 작전'을 설명합니다 — 북방의 교향곡과 바벨탑이 인프라라면, 마레아는 특정 선거를 겨냥해 그 인프라 전체를 가동시키는 실행 단계입니다. 특정 정당이나 후보는 언급하지 않고, 기법 자체에 초점을 맞춥니다.</t>
         </is>
       </c>
     </row>
@@ -22228,10 +22228,10 @@
         </is>
       </c>
       <c r="E691" s="13" t="n">
-        <v>12996</v>
+        <v>12985</v>
       </c>
       <c r="F691" s="13" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G691" s="15" t="inlineStr">
         <is>
@@ -22256,7 +22256,7 @@
         </is>
       </c>
       <c r="E692" s="13" t="n">
-        <v>13018</v>
+        <v>13006</v>
       </c>
       <c r="F692" s="13" t="n">
         <v>19</v>
@@ -22284,10 +22284,10 @@
         </is>
       </c>
       <c r="E693" s="13" t="n">
-        <v>13040</v>
+        <v>13028</v>
       </c>
       <c r="F693" s="13" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G693" s="15" t="inlineStr">
         <is>
@@ -22312,7 +22312,7 @@
         </is>
       </c>
       <c r="E694" s="13" t="n">
-        <v>13062</v>
+        <v>13049</v>
       </c>
       <c r="F694" s="13" t="n">
         <v>18</v>
@@ -22340,7 +22340,7 @@
         </is>
       </c>
       <c r="E695" s="13" t="n">
-        <v>13083</v>
+        <v>13070</v>
       </c>
       <c r="F695" s="13" t="n">
         <v>18</v>
@@ -22368,7 +22368,7 @@
         </is>
       </c>
       <c r="E696" s="13" t="n">
-        <v>13104</v>
+        <v>13091</v>
       </c>
       <c r="F696" s="13" t="n">
         <v>18</v>
@@ -22396,10 +22396,10 @@
         </is>
       </c>
       <c r="E697" s="13" t="n">
-        <v>13125</v>
+        <v>13112</v>
       </c>
       <c r="F697" s="13" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G697" s="15" t="inlineStr">
         <is>
@@ -22424,7 +22424,7 @@
         </is>
       </c>
       <c r="E698" s="13" t="n">
-        <v>13145</v>
+        <v>13134</v>
       </c>
       <c r="F698" s="13" t="n">
         <v>18</v>
@@ -22452,7 +22452,7 @@
         </is>
       </c>
       <c r="E699" s="13" t="n">
-        <v>13166</v>
+        <v>13155</v>
       </c>
       <c r="F699" s="13" t="n">
         <v>17</v>
@@ -22480,7 +22480,7 @@
         </is>
       </c>
       <c r="E700" s="13" t="n">
-        <v>13186</v>
+        <v>13175</v>
       </c>
       <c r="F700" s="13" t="n">
         <v>19</v>
@@ -22508,14 +22508,14 @@
         </is>
       </c>
       <c r="E701" s="13" t="n">
-        <v>13208</v>
+        <v>13197</v>
       </c>
       <c r="F701" s="13" t="n">
         <v>25</v>
       </c>
       <c r="G701" s="15" t="inlineStr">
         <is>
-          <t>새로운 세션. 빅토르가 '돈키호테 작전'을 밝히기 전, 유독 무거운 표정으로 망설입니다. 알바로 가 지금까지 겪었던 '아슬아슬한 추적'들이 사실은 의도된 기만이었다는 사실이 드러나기 시작 합니다.</t>
+          <t>새로운 세션. 빅토르가 '돈키호테 작전'을 밝히기 전, 유독 무거운 표정으로 망설입니다. 알바로가 지금까지 겪었던 '아슬아슬한 추적'들이 사실은 의도된 기만이었다는 사실이 드러나기 시작 합니다.</t>
         </is>
       </c>
     </row>
@@ -22536,10 +22536,10 @@
         </is>
       </c>
       <c r="E702" s="13" t="n">
-        <v>13237</v>
+        <v>13225</v>
       </c>
       <c r="F702" s="13" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G702" s="15" t="inlineStr">
         <is>
@@ -22564,10 +22564,10 @@
         </is>
       </c>
       <c r="E703" s="13" t="n">
-        <v>13257</v>
+        <v>13246</v>
       </c>
       <c r="F703" s="13" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G703" s="15" t="inlineStr">
         <is>
@@ -22592,7 +22592,7 @@
         </is>
       </c>
       <c r="E704" s="13" t="n">
-        <v>13275</v>
+        <v>13263</v>
       </c>
       <c r="F704" s="13" t="n">
         <v>20</v>
@@ -22620,10 +22620,10 @@
         </is>
       </c>
       <c r="E705" s="13" t="n">
-        <v>13298</v>
+        <v>13286</v>
       </c>
       <c r="F705" s="13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G705" s="15" t="inlineStr">
         <is>
@@ -22648,10 +22648,10 @@
         </is>
       </c>
       <c r="E706" s="13" t="n">
-        <v>13318</v>
+        <v>13305</v>
       </c>
       <c r="F706" s="13" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G706" s="15" t="inlineStr">
         <is>
@@ -22676,7 +22676,7 @@
         </is>
       </c>
       <c r="E707" s="13" t="n">
-        <v>13339</v>
+        <v>13325</v>
       </c>
       <c r="F707" s="13" t="n">
         <v>18</v>
@@ -22704,7 +22704,7 @@
         </is>
       </c>
       <c r="E708" s="13" t="n">
-        <v>13360</v>
+        <v>13346</v>
       </c>
       <c r="F708" s="13" t="n">
         <v>18</v>
@@ -22732,7 +22732,7 @@
         </is>
       </c>
       <c r="E709" s="13" t="n">
-        <v>13381</v>
+        <v>13367</v>
       </c>
       <c r="F709" s="13" t="n">
         <v>17</v>
@@ -22760,7 +22760,7 @@
         </is>
       </c>
       <c r="E710" s="13" t="n">
-        <v>13401</v>
+        <v>13387</v>
       </c>
       <c r="F710" s="13" t="n">
         <v>26</v>
@@ -22788,7 +22788,7 @@
         </is>
       </c>
       <c r="E711" s="13" t="n">
-        <v>13430</v>
+        <v>13416</v>
       </c>
       <c r="F711" s="13" t="n">
         <v>28</v>
@@ -22816,10 +22816,10 @@
         </is>
       </c>
       <c r="E712" s="13" t="n">
-        <v>13461</v>
+        <v>13447</v>
       </c>
       <c r="F712" s="13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G712" s="15" t="inlineStr">
         <is>
@@ -22844,7 +22844,7 @@
         </is>
       </c>
       <c r="E713" s="13" t="n">
-        <v>13481</v>
+        <v>13466</v>
       </c>
       <c r="F713" s="13" t="n">
         <v>16</v>
@@ -22872,7 +22872,7 @@
         </is>
       </c>
       <c r="E714" s="13" t="n">
-        <v>13500</v>
+        <v>13485</v>
       </c>
       <c r="F714" s="13" t="n">
         <v>16</v>
@@ -22900,10 +22900,10 @@
         </is>
       </c>
       <c r="E715" s="13" t="n">
-        <v>13519</v>
+        <v>13504</v>
       </c>
       <c r="F715" s="13" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G715" s="15" t="inlineStr">
         <is>
@@ -22928,7 +22928,7 @@
         </is>
       </c>
       <c r="E716" s="13" t="n">
-        <v>13543</v>
+        <v>13527</v>
       </c>
       <c r="F716" s="13" t="n">
         <v>17</v>
@@ -22956,7 +22956,7 @@
         </is>
       </c>
       <c r="E717" s="13" t="n">
-        <v>13563</v>
+        <v>13547</v>
       </c>
       <c r="F717" s="13" t="n">
         <v>16</v>
@@ -22984,7 +22984,7 @@
         </is>
       </c>
       <c r="E718" s="13" t="n">
-        <v>13582</v>
+        <v>13566</v>
       </c>
       <c r="F718" s="13" t="n">
         <v>17</v>
@@ -23012,10 +23012,10 @@
         </is>
       </c>
       <c r="E719" s="13" t="n">
-        <v>13602</v>
+        <v>13586</v>
       </c>
       <c r="F719" s="13" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G719" s="15" t="inlineStr">
         <is>
@@ -23040,10 +23040,10 @@
         </is>
       </c>
       <c r="E720" s="13" t="n">
-        <v>13620</v>
+        <v>13606</v>
       </c>
       <c r="F720" s="13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G720" s="15" t="inlineStr">
         <is>
@@ -23068,7 +23068,7 @@
         </is>
       </c>
       <c r="E721" s="13" t="n">
-        <v>13634</v>
+        <v>13619</v>
       </c>
       <c r="F721" s="13" t="n">
         <v>16</v>
@@ -23096,7 +23096,7 @@
         </is>
       </c>
       <c r="E722" s="13" t="n">
-        <v>13653</v>
+        <v>13638</v>
       </c>
       <c r="F722" s="13" t="n">
         <v>17</v>
@@ -23124,7 +23124,7 @@
         </is>
       </c>
       <c r="E723" s="13" t="n">
-        <v>13673</v>
+        <v>13658</v>
       </c>
       <c r="F723" s="13" t="n">
         <v>14</v>
@@ -23152,7 +23152,7 @@
         </is>
       </c>
       <c r="E724" s="13" t="n">
-        <v>13690</v>
+        <v>13675</v>
       </c>
       <c r="F724" s="13" t="n">
         <v>18</v>
@@ -23180,7 +23180,7 @@
         </is>
       </c>
       <c r="E725" s="13" t="n">
-        <v>13711</v>
+        <v>13696</v>
       </c>
       <c r="F725" s="13" t="n">
         <v>17</v>
@@ -23208,7 +23208,7 @@
         </is>
       </c>
       <c r="E726" s="13" t="n">
-        <v>13731</v>
+        <v>13716</v>
       </c>
       <c r="F726" s="13" t="n">
         <v>15</v>
@@ -23236,7 +23236,7 @@
         </is>
       </c>
       <c r="E727" s="13" t="n">
-        <v>13749</v>
+        <v>13734</v>
       </c>
       <c r="F727" s="13" t="n">
         <v>8</v>
@@ -23264,7 +23264,7 @@
         </is>
       </c>
       <c r="E728" s="13" t="n">
-        <v>13759</v>
+        <v>13744</v>
       </c>
       <c r="F728" s="13" t="n">
         <v>14</v>
@@ -23292,10 +23292,10 @@
         </is>
       </c>
       <c r="E729" s="13" t="n">
-        <v>13776</v>
+        <v>13761</v>
       </c>
       <c r="F729" s="13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G729" s="17" t="inlineStr">
         <is>
@@ -23320,7 +23320,7 @@
         </is>
       </c>
       <c r="E730" s="13" t="n">
-        <v>13796</v>
+        <v>13781</v>
       </c>
       <c r="F730" s="13" t="n">
         <v>17</v>
@@ -23348,7 +23348,7 @@
         </is>
       </c>
       <c r="E731" s="13" t="n">
-        <v>13816</v>
+        <v>13801</v>
       </c>
       <c r="F731" s="13" t="n">
         <v>16</v>
@@ -23376,7 +23376,7 @@
         </is>
       </c>
       <c r="E732" s="13" t="n">
-        <v>13835</v>
+        <v>13821</v>
       </c>
       <c r="F732" s="13" t="n">
         <v>7</v>
@@ -23404,7 +23404,7 @@
         </is>
       </c>
       <c r="E733" s="13" t="n">
-        <v>13844</v>
+        <v>13830</v>
       </c>
       <c r="F733" s="13" t="n">
         <v>9</v>
@@ -23432,7 +23432,7 @@
         </is>
       </c>
       <c r="E734" s="13" t="n">
-        <v>13856</v>
+        <v>13842</v>
       </c>
       <c r="F734" s="13" t="n">
         <v>10</v>
@@ -23460,10 +23460,10 @@
         </is>
       </c>
       <c r="E735" s="13" t="n">
-        <v>13868</v>
+        <v>13854</v>
       </c>
       <c r="F735" s="13" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G735" s="15" t="inlineStr">
         <is>
@@ -23488,7 +23488,7 @@
         </is>
       </c>
       <c r="E736" s="13" t="n">
-        <v>13901</v>
+        <v>13885</v>
       </c>
       <c r="F736" s="13" t="n">
         <v>17</v>
@@ -23516,10 +23516,10 @@
         </is>
       </c>
       <c r="E737" s="13" t="n">
-        <v>13921</v>
+        <v>13905</v>
       </c>
       <c r="F737" s="13" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G737" s="15" t="inlineStr">
         <is>
@@ -23544,7 +23544,7 @@
         </is>
       </c>
       <c r="E738" s="13" t="n">
-        <v>13940</v>
+        <v>13926</v>
       </c>
       <c r="F738" s="13" t="n">
         <v>18</v>
@@ -23572,7 +23572,7 @@
         </is>
       </c>
       <c r="E739" s="13" t="n">
-        <v>13961</v>
+        <v>13947</v>
       </c>
       <c r="F739" s="13" t="n">
         <v>11</v>
@@ -23600,7 +23600,7 @@
         </is>
       </c>
       <c r="E740" s="13" t="n">
-        <v>13974</v>
+        <v>13960</v>
       </c>
       <c r="F740" s="13" t="n">
         <v>18</v>
@@ -23628,7 +23628,7 @@
         </is>
       </c>
       <c r="E741" s="13" t="n">
-        <v>13995</v>
+        <v>13981</v>
       </c>
       <c r="F741" s="13" t="n">
         <v>9</v>
@@ -23656,7 +23656,7 @@
         </is>
       </c>
       <c r="E742" s="13" t="n">
-        <v>14007</v>
+        <v>13993</v>
       </c>
       <c r="F742" s="13" t="n">
         <v>10</v>
@@ -23684,7 +23684,7 @@
         </is>
       </c>
       <c r="E743" s="13" t="n">
-        <v>14019</v>
+        <v>14005</v>
       </c>
       <c r="F743" s="13" t="n">
         <v>10</v>
@@ -23712,10 +23712,10 @@
         </is>
       </c>
       <c r="E744" s="13" t="n">
-        <v>14032</v>
+        <v>14018</v>
       </c>
       <c r="F744" s="13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G744" s="15" t="inlineStr">
         <is>
@@ -23740,10 +23740,10 @@
         </is>
       </c>
       <c r="E745" s="13" t="n">
-        <v>14055</v>
+        <v>14042</v>
       </c>
       <c r="F745" s="13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G745" s="15" t="inlineStr">
         <is>
@@ -23768,7 +23768,7 @@
         </is>
       </c>
       <c r="E746" s="13" t="n">
-        <v>14067</v>
+        <v>14056</v>
       </c>
       <c r="F746" s="13" t="n">
         <v>9</v>
@@ -23796,7 +23796,7 @@
         </is>
       </c>
       <c r="E747" s="13" t="n">
-        <v>14078</v>
+        <v>14067</v>
       </c>
       <c r="F747" s="13" t="n">
         <v>10</v>
@@ -23824,10 +23824,10 @@
         </is>
       </c>
       <c r="E748" s="13" t="n">
-        <v>14091</v>
+        <v>14080</v>
       </c>
       <c r="F748" s="13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G748" s="15" t="inlineStr">
         <is>
@@ -23852,10 +23852,10 @@
         </is>
       </c>
       <c r="E749" s="13" t="n">
-        <v>14105</v>
+        <v>14093</v>
       </c>
       <c r="F749" s="13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G749" s="15" t="inlineStr">
         <is>
@@ -23880,7 +23880,7 @@
         </is>
       </c>
       <c r="E750" s="13" t="n">
-        <v>14136</v>
+        <v>14125</v>
       </c>
       <c r="F750" s="13" t="n">
         <v>16</v>
@@ -23908,7 +23908,7 @@
         </is>
       </c>
       <c r="E751" s="13" t="n">
-        <v>14155</v>
+        <v>14144</v>
       </c>
       <c r="F751" s="13" t="n">
         <v>15</v>
@@ -23936,7 +23936,7 @@
         </is>
       </c>
       <c r="E752" s="13" t="n">
-        <v>14173</v>
+        <v>14162</v>
       </c>
       <c r="F752" s="13" t="n">
         <v>15</v>
@@ -23964,7 +23964,7 @@
         </is>
       </c>
       <c r="E753" s="13" t="n">
-        <v>14191</v>
+        <v>14181</v>
       </c>
       <c r="F753" s="13" t="n">
         <v>9</v>
@@ -23992,7 +23992,7 @@
         </is>
       </c>
       <c r="E754" s="13" t="n">
-        <v>14203</v>
+        <v>14193</v>
       </c>
       <c r="F754" s="13" t="n">
         <v>15</v>
@@ -24020,7 +24020,7 @@
         </is>
       </c>
       <c r="E755" s="13" t="n">
-        <v>14221</v>
+        <v>14211</v>
       </c>
       <c r="F755" s="13" t="n">
         <v>8</v>
@@ -24048,7 +24048,7 @@
         </is>
       </c>
       <c r="E756" s="13" t="n">
-        <v>14231</v>
+        <v>14221</v>
       </c>
       <c r="F756" s="13" t="n">
         <v>9</v>
@@ -24076,7 +24076,7 @@
         </is>
       </c>
       <c r="E757" s="13" t="n">
-        <v>14245</v>
+        <v>14235</v>
       </c>
       <c r="F757" s="13" t="n">
         <v>17</v>
@@ -24104,7 +24104,7 @@
         </is>
       </c>
       <c r="E758" s="13" t="n">
-        <v>14265</v>
+        <v>14255</v>
       </c>
       <c r="F758" s="13" t="n">
         <v>7</v>
@@ -24132,7 +24132,7 @@
         </is>
       </c>
       <c r="E759" s="13" t="n">
-        <v>14274</v>
+        <v>14264</v>
       </c>
       <c r="F759" s="13" t="n">
         <v>10</v>
@@ -24160,7 +24160,7 @@
         </is>
       </c>
       <c r="E760" s="13" t="n">
-        <v>14287</v>
+        <v>14277</v>
       </c>
       <c r="F760" s="13" t="n">
         <v>8</v>
@@ -24188,7 +24188,7 @@
         </is>
       </c>
       <c r="E761" s="13" t="n">
-        <v>14298</v>
+        <v>14288</v>
       </c>
       <c r="F761" s="13" t="n">
         <v>10</v>
@@ -24216,7 +24216,7 @@
         </is>
       </c>
       <c r="E762" s="13" t="n">
-        <v>14310</v>
+        <v>14300</v>
       </c>
       <c r="F762" s="13" t="n">
         <v>9</v>
@@ -24244,7 +24244,7 @@
         </is>
       </c>
       <c r="E763" s="13" t="n">
-        <v>14322</v>
+        <v>14312</v>
       </c>
       <c r="F763" s="13" t="n">
         <v>9</v>
@@ -24272,7 +24272,7 @@
         </is>
       </c>
       <c r="E764" s="13" t="n">
-        <v>14333</v>
+        <v>14323</v>
       </c>
       <c r="F764" s="13" t="n">
         <v>9</v>
@@ -24300,7 +24300,7 @@
         </is>
       </c>
       <c r="E765" s="13" t="n">
-        <v>14345</v>
+        <v>14335</v>
       </c>
       <c r="F765" s="13" t="n">
         <v>8</v>
@@ -24328,7 +24328,7 @@
         </is>
       </c>
       <c r="E766" s="13" t="n">
-        <v>14355</v>
+        <v>14345</v>
       </c>
       <c r="F766" s="13" t="n">
         <v>8</v>
@@ -24356,7 +24356,7 @@
         </is>
       </c>
       <c r="E767" s="13" t="n">
-        <v>14365</v>
+        <v>14355</v>
       </c>
       <c r="F767" s="13" t="n">
         <v>8</v>
@@ -24384,7 +24384,7 @@
         </is>
       </c>
       <c r="E768" s="13" t="n">
-        <v>14375</v>
+        <v>14365</v>
       </c>
       <c r="F768" s="13" t="n">
         <v>8</v>
@@ -24412,7 +24412,7 @@
         </is>
       </c>
       <c r="E769" s="13" t="n">
-        <v>14385</v>
+        <v>14375</v>
       </c>
       <c r="F769" s="13" t="n">
         <v>10</v>
@@ -24440,7 +24440,7 @@
         </is>
       </c>
       <c r="E770" s="13" t="n">
-        <v>14398</v>
+        <v>14388</v>
       </c>
       <c r="F770" s="13" t="n">
         <v>9</v>
@@ -24468,7 +24468,7 @@
         </is>
       </c>
       <c r="E771" s="13" t="n">
-        <v>14409</v>
+        <v>14399</v>
       </c>
       <c r="F771" s="13" t="n">
         <v>9</v>
@@ -24496,7 +24496,7 @@
         </is>
       </c>
       <c r="E772" s="13" t="n">
-        <v>14421</v>
+        <v>14411</v>
       </c>
       <c r="F772" s="13" t="n">
         <v>7</v>
@@ -24524,7 +24524,7 @@
         </is>
       </c>
       <c r="E773" s="13" t="n">
-        <v>14430</v>
+        <v>14420</v>
       </c>
       <c r="F773" s="13" t="n">
         <v>8</v>
@@ -24552,7 +24552,7 @@
         </is>
       </c>
       <c r="E774" s="13" t="n">
-        <v>14441</v>
+        <v>14431</v>
       </c>
       <c r="F774" s="13" t="n">
         <v>8</v>
@@ -24580,7 +24580,7 @@
         </is>
       </c>
       <c r="E775" s="13" t="n">
-        <v>14451</v>
+        <v>14441</v>
       </c>
       <c r="F775" s="13" t="n">
         <v>6</v>
@@ -24608,7 +24608,7 @@
         </is>
       </c>
       <c r="E776" s="13" t="n">
-        <v>14460</v>
+        <v>14450</v>
       </c>
       <c r="F776" s="13" t="n">
         <v>7</v>
@@ -24636,7 +24636,7 @@
         </is>
       </c>
       <c r="E777" s="13" t="n">
-        <v>14468</v>
+        <v>14458</v>
       </c>
       <c r="F777" s="13" t="n">
         <v>16</v>
@@ -24664,7 +24664,7 @@
         </is>
       </c>
       <c r="E778" s="13" t="n">
-        <v>14487</v>
+        <v>14477</v>
       </c>
       <c r="F778" s="13" t="n">
         <v>8</v>
@@ -24692,7 +24692,7 @@
         </is>
       </c>
       <c r="E779" s="13" t="n">
-        <v>14497</v>
+        <v>14487</v>
       </c>
       <c r="F779" s="13" t="n">
         <v>8</v>
@@ -24720,7 +24720,7 @@
         </is>
       </c>
       <c r="E780" s="13" t="n">
-        <v>14507</v>
+        <v>14497</v>
       </c>
       <c r="F780" s="13" t="n">
         <v>11</v>
@@ -24748,7 +24748,7 @@
         </is>
       </c>
       <c r="E781" s="13" t="n">
-        <v>14521</v>
+        <v>14511</v>
       </c>
       <c r="F781" s="13" t="n">
         <v>8</v>
@@ -24776,7 +24776,7 @@
         </is>
       </c>
       <c r="E782" s="13" t="n">
-        <v>14531</v>
+        <v>14521</v>
       </c>
       <c r="F782" s="13" t="n">
         <v>9</v>
@@ -24804,7 +24804,7 @@
         </is>
       </c>
       <c r="E783" s="13" t="n">
-        <v>14543</v>
+        <v>14533</v>
       </c>
       <c r="F783" s="13" t="n">
         <v>8</v>
@@ -24832,7 +24832,7 @@
         </is>
       </c>
       <c r="E784" s="13" t="n">
-        <v>14553</v>
+        <v>14543</v>
       </c>
       <c r="F784" s="13" t="n">
         <v>8</v>
@@ -24860,7 +24860,7 @@
         </is>
       </c>
       <c r="E785" s="13" t="n">
-        <v>14564</v>
+        <v>14554</v>
       </c>
       <c r="F785" s="13" t="n">
         <v>8</v>
@@ -24888,7 +24888,7 @@
         </is>
       </c>
       <c r="E786" s="13" t="n">
-        <v>14574</v>
+        <v>14564</v>
       </c>
       <c r="F786" s="13" t="n">
         <v>8</v>
@@ -24916,7 +24916,7 @@
         </is>
       </c>
       <c r="E787" s="13" t="n">
-        <v>14585</v>
+        <v>14575</v>
       </c>
       <c r="F787" s="13" t="n">
         <v>8</v>
@@ -24944,7 +24944,7 @@
         </is>
       </c>
       <c r="E788" s="13" t="n">
-        <v>14595</v>
+        <v>14585</v>
       </c>
       <c r="F788" s="13" t="n">
         <v>8</v>
@@ -24972,7 +24972,7 @@
         </is>
       </c>
       <c r="E789" s="13" t="n">
-        <v>14606</v>
+        <v>14596</v>
       </c>
       <c r="F789" s="13" t="n">
         <v>8</v>
@@ -25000,7 +25000,7 @@
         </is>
       </c>
       <c r="E790" s="13" t="n">
-        <v>14616</v>
+        <v>14606</v>
       </c>
       <c r="F790" s="13" t="n">
         <v>8</v>
@@ -25028,7 +25028,7 @@
         </is>
       </c>
       <c r="E791" s="13" t="n">
-        <v>14627</v>
+        <v>14617</v>
       </c>
       <c r="F791" s="13" t="n">
         <v>8</v>
@@ -25056,7 +25056,7 @@
         </is>
       </c>
       <c r="E792" s="13" t="n">
-        <v>14637</v>
+        <v>14627</v>
       </c>
       <c r="F792" s="13" t="n">
         <v>8</v>
@@ -25084,7 +25084,7 @@
         </is>
       </c>
       <c r="E793" s="13" t="n">
-        <v>14648</v>
+        <v>14638</v>
       </c>
       <c r="F793" s="13" t="n">
         <v>6</v>
@@ -25112,7 +25112,7 @@
         </is>
       </c>
       <c r="E794" s="13" t="n">
-        <v>14656</v>
+        <v>14646</v>
       </c>
       <c r="F794" s="13" t="n">
         <v>8</v>
@@ -25140,7 +25140,7 @@
         </is>
       </c>
       <c r="E795" s="13" t="n">
-        <v>14667</v>
+        <v>14657</v>
       </c>
       <c r="F795" s="13" t="n">
         <v>8</v>
@@ -25168,7 +25168,7 @@
         </is>
       </c>
       <c r="E796" s="13" t="n">
-        <v>14677</v>
+        <v>14667</v>
       </c>
       <c r="F796" s="13" t="n">
         <v>9</v>
@@ -25196,7 +25196,7 @@
         </is>
       </c>
       <c r="E797" s="13" t="n">
-        <v>14689</v>
+        <v>14679</v>
       </c>
       <c r="F797" s="13" t="n">
         <v>9</v>
@@ -25224,7 +25224,7 @@
         </is>
       </c>
       <c r="E798" s="13" t="n">
-        <v>14700</v>
+        <v>14690</v>
       </c>
       <c r="F798" s="13" t="n">
         <v>9</v>
@@ -25252,7 +25252,7 @@
         </is>
       </c>
       <c r="E799" s="13" t="n">
-        <v>14712</v>
+        <v>14702</v>
       </c>
       <c r="F799" s="13" t="n">
         <v>8</v>
@@ -25280,7 +25280,7 @@
         </is>
       </c>
       <c r="E800" s="13" t="n">
-        <v>14722</v>
+        <v>14712</v>
       </c>
       <c r="F800" s="13" t="n">
         <v>5</v>
@@ -25308,7 +25308,7 @@
         </is>
       </c>
       <c r="E801" s="13" t="n">
-        <v>14730</v>
+        <v>14720</v>
       </c>
       <c r="F801" s="13" t="n">
         <v>13</v>
@@ -25336,7 +25336,7 @@
         </is>
       </c>
       <c r="E802" s="13" t="n">
-        <v>14745</v>
+        <v>14735</v>
       </c>
       <c r="F802" s="13" t="n">
         <v>17</v>
@@ -25364,7 +25364,7 @@
         </is>
       </c>
       <c r="E803" s="13" t="n">
-        <v>14765</v>
+        <v>14755</v>
       </c>
       <c r="F803" s="13" t="n">
         <v>8</v>
@@ -25392,7 +25392,7 @@
         </is>
       </c>
       <c r="E804" s="13" t="n">
-        <v>14776</v>
+        <v>14766</v>
       </c>
       <c r="F804" s="13" t="n">
         <v>8</v>
@@ -25420,7 +25420,7 @@
         </is>
       </c>
       <c r="E805" s="13" t="n">
-        <v>14786</v>
+        <v>14776</v>
       </c>
       <c r="F805" s="13" t="n">
         <v>13</v>
@@ -25448,7 +25448,7 @@
         </is>
       </c>
       <c r="E806" s="13" t="n">
-        <v>14802</v>
+        <v>14792</v>
       </c>
       <c r="F806" s="13" t="n">
         <v>9</v>
@@ -25476,7 +25476,7 @@
         </is>
       </c>
       <c r="E807" s="13" t="n">
-        <v>14813</v>
+        <v>14803</v>
       </c>
       <c r="F807" s="13" t="n">
         <v>7</v>
@@ -25504,7 +25504,7 @@
         </is>
       </c>
       <c r="E808" s="13" t="n">
-        <v>14822</v>
+        <v>14812</v>
       </c>
       <c r="F808" s="13" t="n">
         <v>9</v>
@@ -25532,7 +25532,7 @@
         </is>
       </c>
       <c r="E809" s="13" t="n">
-        <v>14834</v>
+        <v>14824</v>
       </c>
       <c r="F809" s="13" t="n">
         <v>12</v>
@@ -25560,7 +25560,7 @@
         </is>
       </c>
       <c r="E810" s="13" t="n">
-        <v>14848</v>
+        <v>14838</v>
       </c>
       <c r="F810" s="13" t="n">
         <v>11</v>
@@ -25588,7 +25588,7 @@
         </is>
       </c>
       <c r="E811" s="13" t="n">
-        <v>14862</v>
+        <v>14852</v>
       </c>
       <c r="F811" s="13" t="n">
         <v>10</v>
@@ -25616,7 +25616,7 @@
         </is>
       </c>
       <c r="E812" s="13" t="n">
-        <v>14875</v>
+        <v>14865</v>
       </c>
       <c r="F812" s="13" t="n">
         <v>10</v>
@@ -25644,7 +25644,7 @@
         </is>
       </c>
       <c r="E813" s="13" t="n">
-        <v>14887</v>
+        <v>14877</v>
       </c>
       <c r="F813" s="13" t="n">
         <v>11</v>
@@ -25672,7 +25672,7 @@
         </is>
       </c>
       <c r="E814" s="13" t="n">
-        <v>14901</v>
+        <v>14891</v>
       </c>
       <c r="F814" s="13" t="n">
         <v>11</v>
@@ -25700,7 +25700,7 @@
         </is>
       </c>
       <c r="E815" s="13" t="n">
-        <v>14915</v>
+        <v>14905</v>
       </c>
       <c r="F815" s="13" t="n">
         <v>9</v>
@@ -25728,7 +25728,7 @@
         </is>
       </c>
       <c r="E816" s="13" t="n">
-        <v>14926</v>
+        <v>14916</v>
       </c>
       <c r="F816" s="13" t="n">
         <v>11</v>
@@ -25756,7 +25756,7 @@
         </is>
       </c>
       <c r="E817" s="13" t="n">
-        <v>14939</v>
+        <v>14929</v>
       </c>
       <c r="F817" s="13" t="n">
         <v>10</v>
@@ -25784,7 +25784,7 @@
         </is>
       </c>
       <c r="E818" s="13" t="n">
-        <v>14952</v>
+        <v>14942</v>
       </c>
       <c r="F818" s="13" t="n">
         <v>9</v>
@@ -25812,7 +25812,7 @@
         </is>
       </c>
       <c r="E819" s="13" t="n">
-        <v>14963</v>
+        <v>14953</v>
       </c>
       <c r="F819" s="13" t="n">
         <v>9</v>
@@ -25840,7 +25840,7 @@
         </is>
       </c>
       <c r="E820" s="13" t="n">
-        <v>14975</v>
+        <v>14965</v>
       </c>
       <c r="F820" s="13" t="n">
         <v>10</v>
@@ -25868,7 +25868,7 @@
         </is>
       </c>
       <c r="E821" s="13" t="n">
-        <v>14988</v>
+        <v>14978</v>
       </c>
       <c r="F821" s="13" t="n">
         <v>15</v>
@@ -25896,7 +25896,7 @@
         </is>
       </c>
       <c r="E822" s="13" t="n">
-        <v>15005</v>
+        <v>14995</v>
       </c>
       <c r="F822" s="13" t="n">
         <v>16</v>
@@ -25924,7 +25924,7 @@
         </is>
       </c>
       <c r="E823" s="13" t="n">
-        <v>15024</v>
+        <v>15014</v>
       </c>
       <c r="F823" s="13" t="n">
         <v>10</v>
@@ -25952,7 +25952,7 @@
         </is>
       </c>
       <c r="E824" s="13" t="n">
-        <v>15036</v>
+        <v>15026</v>
       </c>
       <c r="F824" s="13" t="n">
         <v>9</v>
@@ -25980,7 +25980,7 @@
         </is>
       </c>
       <c r="E825" s="13" t="n">
-        <v>15048</v>
+        <v>15038</v>
       </c>
       <c r="F825" s="13" t="n">
         <v>8</v>
@@ -26008,7 +26008,7 @@
         </is>
       </c>
       <c r="E826" s="13" t="n">
-        <v>15058</v>
+        <v>15048</v>
       </c>
       <c r="F826" s="13" t="n">
         <v>8</v>
@@ -26036,7 +26036,7 @@
         </is>
       </c>
       <c r="E827" s="13" t="n">
-        <v>15069</v>
+        <v>15059</v>
       </c>
       <c r="F827" s="13" t="n">
         <v>8</v>
@@ -26064,7 +26064,7 @@
         </is>
       </c>
       <c r="E828" s="13" t="n">
-        <v>15079</v>
+        <v>15069</v>
       </c>
       <c r="F828" s="13" t="n">
         <v>9</v>
@@ -26092,7 +26092,7 @@
         </is>
       </c>
       <c r="E829" s="13" t="n">
-        <v>15091</v>
+        <v>15081</v>
       </c>
       <c r="F829" s="13" t="n">
         <v>8</v>
@@ -26120,7 +26120,7 @@
         </is>
       </c>
       <c r="E830" s="13" t="n">
-        <v>15101</v>
+        <v>15091</v>
       </c>
       <c r="F830" s="13" t="n">
         <v>8</v>
@@ -26148,7 +26148,7 @@
         </is>
       </c>
       <c r="E831" s="13" t="n">
-        <v>15112</v>
+        <v>15102</v>
       </c>
       <c r="F831" s="13" t="n">
         <v>8</v>
@@ -26176,7 +26176,7 @@
         </is>
       </c>
       <c r="E832" s="13" t="n">
-        <v>15122</v>
+        <v>15112</v>
       </c>
       <c r="F832" s="13" t="n">
         <v>8</v>
@@ -26204,7 +26204,7 @@
         </is>
       </c>
       <c r="E833" s="13" t="n">
-        <v>15133</v>
+        <v>15123</v>
       </c>
       <c r="F833" s="13" t="n">
         <v>8</v>
@@ -26232,7 +26232,7 @@
         </is>
       </c>
       <c r="E834" s="13" t="n">
-        <v>15143</v>
+        <v>15133</v>
       </c>
       <c r="F834" s="13" t="n">
         <v>8</v>
@@ -26260,7 +26260,7 @@
         </is>
       </c>
       <c r="E835" s="13" t="n">
-        <v>15154</v>
+        <v>15144</v>
       </c>
       <c r="F835" s="13" t="n">
         <v>8</v>
@@ -26288,7 +26288,7 @@
         </is>
       </c>
       <c r="E836" s="13" t="n">
-        <v>15164</v>
+        <v>15154</v>
       </c>
       <c r="F836" s="13" t="n">
         <v>8</v>
@@ -26316,7 +26316,7 @@
         </is>
       </c>
       <c r="E837" s="13" t="n">
-        <v>15175</v>
+        <v>15165</v>
       </c>
       <c r="F837" s="13" t="n">
         <v>7</v>
@@ -26344,7 +26344,7 @@
         </is>
       </c>
       <c r="E838" s="13" t="n">
-        <v>15184</v>
+        <v>15174</v>
       </c>
       <c r="F838" s="13" t="n">
         <v>8</v>
@@ -26372,7 +26372,7 @@
         </is>
       </c>
       <c r="E839" s="13" t="n">
-        <v>15195</v>
+        <v>15185</v>
       </c>
       <c r="F839" s="13" t="n">
         <v>7</v>
@@ -26400,7 +26400,7 @@
         </is>
       </c>
       <c r="E840" s="13" t="n">
-        <v>15204</v>
+        <v>15194</v>
       </c>
       <c r="F840" s="13" t="n">
         <v>6</v>
@@ -26428,7 +26428,7 @@
         </is>
       </c>
       <c r="E841" s="13" t="n">
-        <v>15213</v>
+        <v>15203</v>
       </c>
       <c r="F841" s="13" t="n">
         <v>8</v>
@@ -26456,7 +26456,7 @@
         </is>
       </c>
       <c r="E842" s="13" t="n">
-        <v>15223</v>
+        <v>15213</v>
       </c>
       <c r="F842" s="13" t="n">
         <v>15</v>
@@ -26484,7 +26484,7 @@
         </is>
       </c>
       <c r="E843" s="13" t="n">
-        <v>15241</v>
+        <v>15231</v>
       </c>
       <c r="F843" s="13" t="n">
         <v>9</v>
@@ -26512,7 +26512,7 @@
         </is>
       </c>
       <c r="E844" s="13" t="n">
-        <v>15253</v>
+        <v>15243</v>
       </c>
       <c r="F844" s="13" t="n">
         <v>9</v>
@@ -26540,7 +26540,7 @@
         </is>
       </c>
       <c r="E845" s="13" t="n">
-        <v>15264</v>
+        <v>15254</v>
       </c>
       <c r="F845" s="13" t="n">
         <v>9</v>
@@ -26568,7 +26568,7 @@
         </is>
       </c>
       <c r="E846" s="13" t="n">
-        <v>15276</v>
+        <v>15266</v>
       </c>
       <c r="F846" s="13" t="n">
         <v>8</v>
@@ -26596,7 +26596,7 @@
         </is>
       </c>
       <c r="E847" s="13" t="n">
-        <v>15286</v>
+        <v>15276</v>
       </c>
       <c r="F847" s="13" t="n">
         <v>8</v>
@@ -26624,7 +26624,7 @@
         </is>
       </c>
       <c r="E848" s="13" t="n">
-        <v>15297</v>
+        <v>15287</v>
       </c>
       <c r="F848" s="13" t="n">
         <v>9</v>
@@ -26652,7 +26652,7 @@
         </is>
       </c>
       <c r="E849" s="13" t="n">
-        <v>15308</v>
+        <v>15298</v>
       </c>
       <c r="F849" s="13" t="n">
         <v>9</v>
@@ -26680,7 +26680,7 @@
         </is>
       </c>
       <c r="E850" s="13" t="n">
-        <v>15320</v>
+        <v>15310</v>
       </c>
       <c r="F850" s="13" t="n">
         <v>8</v>
@@ -26708,7 +26708,7 @@
         </is>
       </c>
       <c r="E851" s="13" t="n">
-        <v>15330</v>
+        <v>15320</v>
       </c>
       <c r="F851" s="13" t="n">
         <v>9</v>
@@ -26736,7 +26736,7 @@
         </is>
       </c>
       <c r="E852" s="13" t="n">
-        <v>15342</v>
+        <v>15332</v>
       </c>
       <c r="F852" s="13" t="n">
         <v>9</v>
@@ -26764,7 +26764,7 @@
         </is>
       </c>
       <c r="E853" s="13" t="n">
-        <v>15353</v>
+        <v>15343</v>
       </c>
       <c r="F853" s="13" t="n">
         <v>9</v>
@@ -26792,7 +26792,7 @@
         </is>
       </c>
       <c r="E854" s="13" t="n">
-        <v>15365</v>
+        <v>15355</v>
       </c>
       <c r="F854" s="13" t="n">
         <v>9</v>
@@ -26820,7 +26820,7 @@
         </is>
       </c>
       <c r="E855" s="13" t="n">
-        <v>15376</v>
+        <v>15366</v>
       </c>
       <c r="F855" s="13" t="n">
         <v>8</v>
@@ -26848,7 +26848,7 @@
         </is>
       </c>
       <c r="E856" s="13" t="n">
-        <v>15387</v>
+        <v>15377</v>
       </c>
       <c r="F856" s="13" t="n">
         <v>7</v>
@@ -26876,7 +26876,7 @@
         </is>
       </c>
       <c r="E857" s="13" t="n">
-        <v>15396</v>
+        <v>15386</v>
       </c>
       <c r="F857" s="13" t="n">
         <v>7</v>
@@ -26904,7 +26904,7 @@
         </is>
       </c>
       <c r="E858" s="13" t="n">
-        <v>15406</v>
+        <v>15396</v>
       </c>
       <c r="F858" s="13" t="n">
         <v>8</v>
@@ -26932,7 +26932,7 @@
         </is>
       </c>
       <c r="E859" s="13" t="n">
-        <v>15416</v>
+        <v>15406</v>
       </c>
       <c r="F859" s="13" t="n">
         <v>9</v>
@@ -26960,7 +26960,7 @@
         </is>
       </c>
       <c r="E860" s="13" t="n">
-        <v>15428</v>
+        <v>15418</v>
       </c>
       <c r="F860" s="13" t="n">
         <v>8</v>
@@ -26988,7 +26988,7 @@
         </is>
       </c>
       <c r="E861" s="13" t="n">
-        <v>15438</v>
+        <v>15428</v>
       </c>
       <c r="F861" s="13" t="n">
         <v>10</v>
@@ -27016,7 +27016,7 @@
         </is>
       </c>
       <c r="E862" s="13" t="n">
-        <v>15451</v>
+        <v>15441</v>
       </c>
       <c r="F862" s="13" t="n">
         <v>9</v>
@@ -27044,7 +27044,7 @@
         </is>
       </c>
       <c r="E863" s="13" t="n">
-        <v>15462</v>
+        <v>15452</v>
       </c>
       <c r="F863" s="13" t="n">
         <v>8</v>
@@ -27072,7 +27072,7 @@
         </is>
       </c>
       <c r="E864" s="13" t="n">
-        <v>15473</v>
+        <v>15463</v>
       </c>
       <c r="F864" s="13" t="n">
         <v>8</v>
@@ -27100,7 +27100,7 @@
         </is>
       </c>
       <c r="E865" s="13" t="n">
-        <v>15483</v>
+        <v>15473</v>
       </c>
       <c r="F865" s="13" t="n">
         <v>7</v>
@@ -27128,7 +27128,7 @@
         </is>
       </c>
       <c r="E866" s="13" t="n">
-        <v>15493</v>
+        <v>15483</v>
       </c>
       <c r="F866" s="13" t="n">
         <v>9</v>
@@ -27156,7 +27156,7 @@
         </is>
       </c>
       <c r="E867" s="13" t="n">
-        <v>15504</v>
+        <v>15494</v>
       </c>
       <c r="F867" s="13" t="n">
         <v>9</v>
@@ -27184,7 +27184,7 @@
         </is>
       </c>
       <c r="E868" s="13" t="n">
-        <v>15516</v>
+        <v>15506</v>
       </c>
       <c r="F868" s="13" t="n">
         <v>8</v>
@@ -27212,7 +27212,7 @@
         </is>
       </c>
       <c r="E869" s="13" t="n">
-        <v>15526</v>
+        <v>15516</v>
       </c>
       <c r="F869" s="13" t="n">
         <v>8</v>
@@ -27240,7 +27240,7 @@
         </is>
       </c>
       <c r="E870" s="13" t="n">
-        <v>15537</v>
+        <v>15527</v>
       </c>
       <c r="F870" s="13" t="n">
         <v>9</v>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="E871" s="13" t="n">
-        <v>15548</v>
+        <v>15538</v>
       </c>
       <c r="F871" s="13" t="n">
         <v>8</v>
@@ -27296,7 +27296,7 @@
         </is>
       </c>
       <c r="E872" s="13" t="n">
-        <v>15559</v>
+        <v>15549</v>
       </c>
       <c r="F872" s="13" t="n">
         <v>8</v>
@@ -27324,7 +27324,7 @@
         </is>
       </c>
       <c r="E873" s="13" t="n">
-        <v>15569</v>
+        <v>15559</v>
       </c>
       <c r="F873" s="13" t="n">
         <v>8</v>
@@ -27352,7 +27352,7 @@
         </is>
       </c>
       <c r="E874" s="13" t="n">
-        <v>15580</v>
+        <v>15570</v>
       </c>
       <c r="F874" s="13" t="n">
         <v>8</v>
@@ -27380,7 +27380,7 @@
         </is>
       </c>
       <c r="E875" s="13" t="n">
-        <v>15590</v>
+        <v>15580</v>
       </c>
       <c r="F875" s="13" t="n">
         <v>8</v>
@@ -27408,7 +27408,7 @@
         </is>
       </c>
       <c r="E876" s="13" t="n">
-        <v>15601</v>
+        <v>15591</v>
       </c>
       <c r="F876" s="13" t="n">
         <v>8</v>
@@ -27436,7 +27436,7 @@
         </is>
       </c>
       <c r="E877" s="13" t="n">
-        <v>15611</v>
+        <v>15601</v>
       </c>
       <c r="F877" s="13" t="n">
         <v>6</v>
@@ -27464,7 +27464,7 @@
         </is>
       </c>
       <c r="E878" s="13" t="n">
-        <v>15620</v>
+        <v>15610</v>
       </c>
       <c r="F878" s="13" t="n">
         <v>7</v>
@@ -27492,7 +27492,7 @@
         </is>
       </c>
       <c r="E879" s="13" t="n">
-        <v>15629</v>
+        <v>15619</v>
       </c>
       <c r="F879" s="13" t="n">
         <v>8</v>
@@ -27520,7 +27520,7 @@
         </is>
       </c>
       <c r="E880" s="13" t="n">
-        <v>15640</v>
+        <v>15630</v>
       </c>
       <c r="F880" s="13" t="n">
         <v>8</v>
@@ -27548,7 +27548,7 @@
         </is>
       </c>
       <c r="E881" s="13" t="n">
-        <v>15650</v>
+        <v>15640</v>
       </c>
       <c r="F881" s="13" t="n">
         <v>9</v>
@@ -27576,7 +27576,7 @@
         </is>
       </c>
       <c r="E882" s="13" t="n">
-        <v>15662</v>
+        <v>15652</v>
       </c>
       <c r="F882" s="13" t="n">
         <v>7</v>
@@ -27604,7 +27604,7 @@
         </is>
       </c>
       <c r="E883" s="13" t="n">
-        <v>15671</v>
+        <v>15661</v>
       </c>
       <c r="F883" s="13" t="n">
         <v>9</v>
@@ -27632,7 +27632,7 @@
         </is>
       </c>
       <c r="E884" s="13" t="n">
-        <v>15683</v>
+        <v>15673</v>
       </c>
       <c r="F884" s="13" t="n">
         <v>8</v>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="E885" s="13" t="n">
-        <v>15693</v>
+        <v>15683</v>
       </c>
       <c r="F885" s="13" t="n">
         <v>6</v>
@@ -27688,7 +27688,7 @@
         </is>
       </c>
       <c r="E886" s="13" t="n">
-        <v>15702</v>
+        <v>15692</v>
       </c>
       <c r="F886" s="13" t="n">
         <v>8</v>
@@ -27716,7 +27716,7 @@
         </is>
       </c>
       <c r="E887" s="13" t="n">
-        <v>15712</v>
+        <v>15702</v>
       </c>
       <c r="F887" s="13" t="n">
         <v>9</v>
@@ -27744,7 +27744,7 @@
         </is>
       </c>
       <c r="E888" s="13" t="n">
-        <v>15724</v>
+        <v>15714</v>
       </c>
       <c r="F888" s="13" t="n">
         <v>7</v>
@@ -27772,7 +27772,7 @@
         </is>
       </c>
       <c r="E889" s="13" t="n">
-        <v>15733</v>
+        <v>15723</v>
       </c>
       <c r="F889" s="13" t="n">
         <v>8</v>
@@ -27800,7 +27800,7 @@
         </is>
       </c>
       <c r="E890" s="13" t="n">
-        <v>15744</v>
+        <v>15734</v>
       </c>
       <c r="F890" s="13" t="n">
         <v>7</v>
@@ -27828,7 +27828,7 @@
         </is>
       </c>
       <c r="E891" s="13" t="n">
-        <v>15753</v>
+        <v>15743</v>
       </c>
       <c r="F891" s="13" t="n">
         <v>7</v>
@@ -27856,7 +27856,7 @@
         </is>
       </c>
       <c r="E892" s="13" t="n">
-        <v>15763</v>
+        <v>15753</v>
       </c>
       <c r="F892" s="13" t="n">
         <v>8</v>
@@ -27884,7 +27884,7 @@
         </is>
       </c>
       <c r="E893" s="13" t="n">
-        <v>15773</v>
+        <v>15763</v>
       </c>
       <c r="F893" s="13" t="n">
         <v>9</v>
@@ -27912,7 +27912,7 @@
         </is>
       </c>
       <c r="E894" s="13" t="n">
-        <v>15785</v>
+        <v>15775</v>
       </c>
       <c r="F894" s="13" t="n">
         <v>8</v>
@@ -27940,7 +27940,7 @@
         </is>
       </c>
       <c r="E895" s="13" t="n">
-        <v>15795</v>
+        <v>15785</v>
       </c>
       <c r="F895" s="13" t="n">
         <v>6</v>
@@ -27968,7 +27968,7 @@
         </is>
       </c>
       <c r="E896" s="13" t="n">
-        <v>15804</v>
+        <v>15794</v>
       </c>
       <c r="F896" s="13" t="n">
         <v>7</v>
@@ -27996,7 +27996,7 @@
         </is>
       </c>
       <c r="E897" s="13" t="n">
-        <v>15813</v>
+        <v>15803</v>
       </c>
       <c r="F897" s="13" t="n">
         <v>8</v>
@@ -28024,7 +28024,7 @@
         </is>
       </c>
       <c r="E898" s="13" t="n">
-        <v>15823</v>
+        <v>15813</v>
       </c>
       <c r="F898" s="13" t="n">
         <v>7</v>
@@ -28052,7 +28052,7 @@
         </is>
       </c>
       <c r="E899" s="13" t="n">
-        <v>15832</v>
+        <v>15822</v>
       </c>
       <c r="F899" s="13" t="n">
         <v>8</v>
@@ -28080,7 +28080,7 @@
         </is>
       </c>
       <c r="E900" s="13" t="n">
-        <v>15842</v>
+        <v>15832</v>
       </c>
       <c r="F900" s="13" t="n">
         <v>8</v>
@@ -28108,7 +28108,7 @@
         </is>
       </c>
       <c r="E901" s="13" t="n">
-        <v>15853</v>
+        <v>15843</v>
       </c>
       <c r="F901" s="13" t="n">
         <v>7</v>
@@ -28136,7 +28136,7 @@
         </is>
       </c>
       <c r="E902" s="13" t="n">
-        <v>15862</v>
+        <v>15852</v>
       </c>
       <c r="F902" s="13" t="n">
         <v>7</v>
@@ -28164,7 +28164,7 @@
         </is>
       </c>
       <c r="E903" s="13" t="n">
-        <v>15872</v>
+        <v>15862</v>
       </c>
       <c r="F903" s="13" t="n">
         <v>7</v>
@@ -28192,7 +28192,7 @@
         </is>
       </c>
       <c r="E904" s="13" t="n">
-        <v>15881</v>
+        <v>15871</v>
       </c>
       <c r="F904" s="13" t="n">
         <v>8</v>
@@ -28220,7 +28220,7 @@
         </is>
       </c>
       <c r="E905" s="13" t="n">
-        <v>15892</v>
+        <v>15882</v>
       </c>
       <c r="F905" s="13" t="n">
         <v>8</v>
@@ -28248,7 +28248,7 @@
         </is>
       </c>
       <c r="E906" s="13" t="n">
-        <v>15902</v>
+        <v>15892</v>
       </c>
       <c r="F906" s="13" t="n">
         <v>8</v>
@@ -28276,7 +28276,7 @@
         </is>
       </c>
       <c r="E907" s="13" t="n">
-        <v>15913</v>
+        <v>15903</v>
       </c>
       <c r="F907" s="13" t="n">
         <v>8</v>
@@ -28304,7 +28304,7 @@
         </is>
       </c>
       <c r="E908" s="13" t="n">
-        <v>15923</v>
+        <v>15913</v>
       </c>
       <c r="F908" s="13" t="n">
         <v>9</v>
@@ -28332,7 +28332,7 @@
         </is>
       </c>
       <c r="E909" s="13" t="n">
-        <v>15935</v>
+        <v>15925</v>
       </c>
       <c r="F909" s="13" t="n">
         <v>9</v>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="E910" s="13" t="n">
-        <v>15946</v>
+        <v>15936</v>
       </c>
       <c r="F910" s="13" t="n">
         <v>9</v>
@@ -28388,7 +28388,7 @@
         </is>
       </c>
       <c r="E911" s="13" t="n">
-        <v>15958</v>
+        <v>15948</v>
       </c>
       <c r="F911" s="13" t="n">
         <v>9</v>
@@ -28416,7 +28416,7 @@
         </is>
       </c>
       <c r="E912" s="13" t="n">
-        <v>15969</v>
+        <v>15959</v>
       </c>
       <c r="F912" s="13" t="n">
         <v>8</v>
@@ -28444,7 +28444,7 @@
         </is>
       </c>
       <c r="E913" s="13" t="n">
-        <v>15980</v>
+        <v>15970</v>
       </c>
       <c r="F913" s="13" t="n">
         <v>7</v>
@@ -28472,7 +28472,7 @@
         </is>
       </c>
       <c r="E914" s="13" t="n">
-        <v>15989</v>
+        <v>15979</v>
       </c>
       <c r="F914" s="13" t="n">
         <v>8</v>
@@ -28500,7 +28500,7 @@
         </is>
       </c>
       <c r="E915" s="13" t="n">
-        <v>16000</v>
+        <v>15990</v>
       </c>
       <c r="F915" s="13" t="n">
         <v>7</v>
@@ -28528,7 +28528,7 @@
         </is>
       </c>
       <c r="E916" s="13" t="n">
-        <v>16009</v>
+        <v>15999</v>
       </c>
       <c r="F916" s="13" t="n">
         <v>7</v>
@@ -28556,7 +28556,7 @@
         </is>
       </c>
       <c r="E917" s="13" t="n">
-        <v>16018</v>
+        <v>16008</v>
       </c>
       <c r="F917" s="13" t="n">
         <v>6</v>
@@ -28584,7 +28584,7 @@
         </is>
       </c>
       <c r="E918" s="13" t="n">
-        <v>16027</v>
+        <v>16017</v>
       </c>
       <c r="F918" s="13" t="n">
         <v>5</v>
@@ -28612,7 +28612,7 @@
         </is>
       </c>
       <c r="E919" s="13" t="n">
-        <v>16034</v>
+        <v>16024</v>
       </c>
       <c r="F919" s="13" t="n">
         <v>7</v>
@@ -28640,7 +28640,7 @@
         </is>
       </c>
       <c r="E920" s="13" t="n">
-        <v>16043</v>
+        <v>16033</v>
       </c>
       <c r="F920" s="13" t="n">
         <v>6</v>
@@ -28668,7 +28668,7 @@
         </is>
       </c>
       <c r="E921" s="13" t="n">
-        <v>16052</v>
+        <v>16042</v>
       </c>
       <c r="F921" s="13" t="n">
         <v>7</v>
@@ -28696,7 +28696,7 @@
         </is>
       </c>
       <c r="E922" s="13" t="n">
-        <v>16061</v>
+        <v>16051</v>
       </c>
       <c r="F922" s="13" t="n">
         <v>8</v>
@@ -28724,7 +28724,7 @@
         </is>
       </c>
       <c r="E923" s="13" t="n">
-        <v>16072</v>
+        <v>16062</v>
       </c>
       <c r="F923" s="13" t="n">
         <v>7</v>
@@ -28752,7 +28752,7 @@
         </is>
       </c>
       <c r="E924" s="13" t="n">
-        <v>16081</v>
+        <v>16071</v>
       </c>
       <c r="F924" s="13" t="n">
         <v>14</v>
@@ -28780,7 +28780,7 @@
         </is>
       </c>
       <c r="E925" s="13" t="n">
-        <v>16098</v>
+        <v>16088</v>
       </c>
       <c r="F925" s="13" t="n">
         <v>7</v>
@@ -28808,7 +28808,7 @@
         </is>
       </c>
       <c r="E926" s="13" t="n">
-        <v>16107</v>
+        <v>16097</v>
       </c>
       <c r="F926" s="13" t="n">
         <v>8</v>
@@ -28836,7 +28836,7 @@
         </is>
       </c>
       <c r="E927" s="13" t="n">
-        <v>16118</v>
+        <v>16108</v>
       </c>
       <c r="F927" s="13" t="n">
         <v>6</v>
@@ -28864,7 +28864,7 @@
         </is>
       </c>
       <c r="E928" s="13" t="n">
-        <v>16126</v>
+        <v>16116</v>
       </c>
       <c r="F928" s="13" t="n">
         <v>7</v>
@@ -28892,7 +28892,7 @@
         </is>
       </c>
       <c r="E929" s="13" t="n">
-        <v>16135</v>
+        <v>16125</v>
       </c>
       <c r="F929" s="13" t="n">
         <v>5</v>
@@ -28920,7 +28920,7 @@
         </is>
       </c>
       <c r="E930" s="13" t="n">
-        <v>16143</v>
+        <v>16133</v>
       </c>
       <c r="F930" s="13" t="n">
         <v>7</v>
@@ -28948,7 +28948,7 @@
         </is>
       </c>
       <c r="E931" s="13" t="n">
-        <v>16152</v>
+        <v>16142</v>
       </c>
       <c r="F931" s="13" t="n">
         <v>7</v>
@@ -28976,7 +28976,7 @@
         </is>
       </c>
       <c r="E932" s="13" t="n">
-        <v>16162</v>
+        <v>16152</v>
       </c>
       <c r="F932" s="13" t="n">
         <v>8</v>
@@ -29004,7 +29004,7 @@
         </is>
       </c>
       <c r="E933" s="13" t="n">
-        <v>16172</v>
+        <v>16162</v>
       </c>
       <c r="F933" s="13" t="n">
         <v>8</v>
@@ -29032,7 +29032,7 @@
         </is>
       </c>
       <c r="E934" s="13" t="n">
-        <v>16183</v>
+        <v>16173</v>
       </c>
       <c r="F934" s="13" t="n">
         <v>7</v>
@@ -29060,7 +29060,7 @@
         </is>
       </c>
       <c r="E935" s="13" t="n">
-        <v>16192</v>
+        <v>16182</v>
       </c>
       <c r="F935" s="13" t="n">
         <v>7</v>
@@ -29088,7 +29088,7 @@
         </is>
       </c>
       <c r="E936" s="13" t="n">
-        <v>16201</v>
+        <v>16191</v>
       </c>
       <c r="F936" s="13" t="n">
         <v>7</v>
@@ -29116,7 +29116,7 @@
         </is>
       </c>
       <c r="E937" s="13" t="n">
-        <v>16210</v>
+        <v>16200</v>
       </c>
       <c r="F937" s="13" t="n">
         <v>5</v>
@@ -29144,7 +29144,7 @@
         </is>
       </c>
       <c r="E938" s="13" t="n">
-        <v>16217</v>
+        <v>16207</v>
       </c>
       <c r="F938" s="13" t="n">
         <v>15</v>
@@ -29172,7 +29172,7 @@
         </is>
       </c>
       <c r="E939" s="13" t="n">
-        <v>16235</v>
+        <v>16225</v>
       </c>
       <c r="F939" s="13" t="n">
         <v>15</v>
@@ -29200,7 +29200,7 @@
         </is>
       </c>
       <c r="E940" s="13" t="n">
-        <v>16253</v>
+        <v>16243</v>
       </c>
       <c r="F940" s="13" t="n">
         <v>8</v>
@@ -29228,7 +29228,7 @@
         </is>
       </c>
       <c r="E941" s="13" t="n">
-        <v>16263</v>
+        <v>16253</v>
       </c>
       <c r="F941" s="13" t="n">
         <v>7</v>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="E942" s="13" t="n">
-        <v>16273</v>
+        <v>16263</v>
       </c>
       <c r="F942" s="13" t="n">
         <v>6</v>
@@ -29284,7 +29284,7 @@
         </is>
       </c>
       <c r="E943" s="13" t="n">
-        <v>16281</v>
+        <v>16271</v>
       </c>
       <c r="F943" s="13" t="n">
         <v>6</v>
@@ -29312,7 +29312,7 @@
         </is>
       </c>
       <c r="E944" s="13" t="n">
-        <v>16289</v>
+        <v>16279</v>
       </c>
       <c r="F944" s="13" t="n">
         <v>7</v>
@@ -29340,7 +29340,7 @@
         </is>
       </c>
       <c r="E945" s="13" t="n">
-        <v>16299</v>
+        <v>16289</v>
       </c>
       <c r="F945" s="13" t="n">
         <v>4</v>
@@ -29368,7 +29368,7 @@
         </is>
       </c>
       <c r="E946" s="13" t="n">
-        <v>16305</v>
+        <v>16295</v>
       </c>
       <c r="F946" s="13" t="n">
         <v>6</v>
@@ -29396,7 +29396,7 @@
         </is>
       </c>
       <c r="E947" s="13" t="n">
-        <v>16313</v>
+        <v>16303</v>
       </c>
       <c r="F947" s="13" t="n">
         <v>7</v>
@@ -29424,7 +29424,7 @@
         </is>
       </c>
       <c r="E948" s="13" t="n">
-        <v>16323</v>
+        <v>16313</v>
       </c>
       <c r="F948" s="13" t="n">
         <v>6</v>
@@ -29452,7 +29452,7 @@
         </is>
       </c>
       <c r="E949" s="13" t="n">
-        <v>16331</v>
+        <v>16321</v>
       </c>
       <c r="F949" s="13" t="n">
         <v>9</v>
@@ -29480,7 +29480,7 @@
         </is>
       </c>
       <c r="E950" s="13" t="n">
-        <v>16343</v>
+        <v>16333</v>
       </c>
       <c r="F950" s="13" t="n">
         <v>6</v>
@@ -29508,7 +29508,7 @@
         </is>
       </c>
       <c r="E951" s="13" t="n">
-        <v>16351</v>
+        <v>16341</v>
       </c>
       <c r="F951" s="13" t="n">
         <v>7</v>
@@ -29536,7 +29536,7 @@
         </is>
       </c>
       <c r="E952" s="13" t="n">
-        <v>16360</v>
+        <v>16350</v>
       </c>
       <c r="F952" s="13" t="n">
         <v>6</v>
@@ -29564,7 +29564,7 @@
         </is>
       </c>
       <c r="E953" s="13" t="n">
-        <v>16368</v>
+        <v>16358</v>
       </c>
       <c r="F953" s="13" t="n">
         <v>6</v>
@@ -29592,7 +29592,7 @@
         </is>
       </c>
       <c r="E954" s="13" t="n">
-        <v>16376</v>
+        <v>16366</v>
       </c>
       <c r="F954" s="13" t="n">
         <v>7</v>
@@ -29620,7 +29620,7 @@
         </is>
       </c>
       <c r="E955" s="13" t="n">
-        <v>16386</v>
+        <v>16376</v>
       </c>
       <c r="F955" s="13" t="n">
         <v>7</v>
@@ -29648,7 +29648,7 @@
         </is>
       </c>
       <c r="E956" s="13" t="n">
-        <v>16395</v>
+        <v>16385</v>
       </c>
       <c r="F956" s="13" t="n">
         <v>7</v>
@@ -29676,7 +29676,7 @@
         </is>
       </c>
       <c r="E957" s="13" t="n">
-        <v>16404</v>
+        <v>16394</v>
       </c>
       <c r="F957" s="13" t="n">
         <v>7</v>
@@ -29704,7 +29704,7 @@
         </is>
       </c>
       <c r="E958" s="13" t="n">
-        <v>16413</v>
+        <v>16403</v>
       </c>
       <c r="F958" s="13" t="n">
         <v>7</v>
@@ -29732,7 +29732,7 @@
         </is>
       </c>
       <c r="E959" s="13" t="n">
-        <v>16422</v>
+        <v>16412</v>
       </c>
       <c r="F959" s="13" t="n">
         <v>5</v>
@@ -29760,7 +29760,7 @@
         </is>
       </c>
       <c r="E960" s="13" t="n">
-        <v>16430</v>
+        <v>16420</v>
       </c>
       <c r="F960" s="13" t="n">
         <v>5</v>
@@ -29788,7 +29788,7 @@
         </is>
       </c>
       <c r="E961" s="13" t="n">
-        <v>16437</v>
+        <v>16427</v>
       </c>
       <c r="F961" s="13" t="n">
         <v>5</v>
@@ -29816,7 +29816,7 @@
         </is>
       </c>
       <c r="E962" s="13" t="n">
-        <v>16445</v>
+        <v>16435</v>
       </c>
       <c r="F962" s="13" t="n">
         <v>6</v>
@@ -29844,7 +29844,7 @@
         </is>
       </c>
       <c r="E963" s="13" t="n">
-        <v>16453</v>
+        <v>16443</v>
       </c>
       <c r="F963" s="13" t="n">
         <v>7</v>
@@ -29872,7 +29872,7 @@
         </is>
       </c>
       <c r="E964" s="13" t="n">
-        <v>16462</v>
+        <v>16452</v>
       </c>
       <c r="F964" s="13" t="n">
         <v>6</v>
@@ -29900,7 +29900,7 @@
         </is>
       </c>
       <c r="E965" s="13" t="n">
-        <v>16470</v>
+        <v>16460</v>
       </c>
       <c r="F965" s="13" t="n">
         <v>7</v>
@@ -29928,7 +29928,7 @@
         </is>
       </c>
       <c r="E966" s="13" t="n">
-        <v>16479</v>
+        <v>16469</v>
       </c>
       <c r="F966" s="13" t="n">
         <v>8</v>
@@ -29956,7 +29956,7 @@
         </is>
       </c>
       <c r="E967" s="13" t="n">
-        <v>16490</v>
+        <v>16480</v>
       </c>
       <c r="F967" s="13" t="n">
         <v>7</v>
@@ -29984,7 +29984,7 @@
         </is>
       </c>
       <c r="E968" s="13" t="n">
-        <v>16499</v>
+        <v>16489</v>
       </c>
       <c r="F968" s="13" t="n">
         <v>6</v>
@@ -30012,7 +30012,7 @@
         </is>
       </c>
       <c r="E969" s="13" t="n">
-        <v>16508</v>
+        <v>16498</v>
       </c>
       <c r="F969" s="13" t="n">
         <v>7</v>
@@ -30040,7 +30040,7 @@
         </is>
       </c>
       <c r="E970" s="13" t="n">
-        <v>16517</v>
+        <v>16507</v>
       </c>
       <c r="F970" s="13" t="n">
         <v>6</v>
@@ -30068,7 +30068,7 @@
         </is>
       </c>
       <c r="E971" s="13" t="n">
-        <v>16525</v>
+        <v>16515</v>
       </c>
       <c r="F971" s="13" t="n">
         <v>7</v>
@@ -30096,7 +30096,7 @@
         </is>
       </c>
       <c r="E972" s="13" t="n">
-        <v>16535</v>
+        <v>16525</v>
       </c>
       <c r="F972" s="13" t="n">
         <v>7</v>
@@ -30124,7 +30124,7 @@
         </is>
       </c>
       <c r="E973" s="13" t="n">
-        <v>16544</v>
+        <v>16534</v>
       </c>
       <c r="F973" s="13" t="n">
         <v>3</v>
@@ -30152,7 +30152,7 @@
         </is>
       </c>
       <c r="E974" s="13" t="n">
-        <v>16550</v>
+        <v>16540</v>
       </c>
       <c r="F974" s="13" t="n">
         <v>2</v>
@@ -30180,7 +30180,7 @@
         </is>
       </c>
       <c r="E975" s="13" t="n">
-        <v>16554</v>
+        <v>16544</v>
       </c>
       <c r="F975" s="13" t="n">
         <v>5</v>
@@ -30208,7 +30208,7 @@
         </is>
       </c>
       <c r="E976" s="13" t="n">
-        <v>16561</v>
+        <v>16551</v>
       </c>
       <c r="F976" s="13" t="n">
         <v>13</v>
@@ -30236,7 +30236,7 @@
         </is>
       </c>
       <c r="E977" s="13" t="n">
-        <v>16577</v>
+        <v>16567</v>
       </c>
       <c r="F977" s="13" t="n">
         <v>24</v>
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="E978" s="13" t="n">
-        <v>16604</v>
+        <v>16594</v>
       </c>
       <c r="F978" s="13" t="n">
         <v>23</v>
@@ -30292,7 +30292,7 @@
         </is>
       </c>
       <c r="E979" s="13" t="n">
-        <v>16631</v>
+        <v>16621</v>
       </c>
       <c r="F979" s="13" t="n">
         <v>19</v>
@@ -30320,7 +30320,7 @@
         </is>
       </c>
       <c r="E980" s="13" t="n">
-        <v>16653</v>
+        <v>16643</v>
       </c>
       <c r="F980" s="13" t="n">
         <v>18</v>
@@ -30348,7 +30348,7 @@
         </is>
       </c>
       <c r="E981" s="13" t="n">
-        <v>16674</v>
+        <v>16664</v>
       </c>
       <c r="F981" s="13" t="n">
         <v>19</v>

</xml_diff>